<commit_message>
feat: apply user overhead rates (Chi phi chung 20%, Thu nhap 5.5%, VAT 8%, Du phong 0%)
</commit_message>
<xml_diff>
--- a/backend/data/DU_TOAN_QUAN_TRAC_MOI_TRUONG_CHUAN_6_SHEET_F1.xlsx
+++ b/backend/data/DU_TOAN_QUAN_TRAC_MOI_TRUONG_CHUAN_6_SHEET_F1.xlsx
@@ -10382,7 +10382,7 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>191100</v>
+        <v>370000</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
@@ -10415,7 +10415,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>235</v>
+        <v>370</v>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
@@ -10547,7 +10547,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>1180</v>
+        <v>59100</v>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
@@ -11240,7 +11240,7 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>191100</v>
+        <v>40000</v>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
@@ -11273,7 +11273,7 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>191100</v>
+        <v>40000</v>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
@@ -11306,7 +11306,7 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>235</v>
+        <v>40</v>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
@@ -11339,7 +11339,7 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>235</v>
+        <v>40</v>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
@@ -11405,7 +11405,7 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>8330</v>
+        <v>4780</v>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
@@ -11603,7 +11603,7 @@
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>8330</v>
+        <v>1920</v>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
@@ -11636,7 +11636,7 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>8330</v>
+        <v>1707</v>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
@@ -11669,7 +11669,7 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>441000</v>
+        <v>853333</v>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
@@ -11702,7 +11702,7 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>274</v>
+        <v>390</v>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
@@ -11735,7 +11735,7 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>274</v>
+        <v>1200</v>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
@@ -11801,7 +11801,7 @@
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>1180</v>
+        <v>12700</v>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
@@ -11834,7 +11834,7 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>274</v>
+        <v>1270</v>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
@@ -11867,7 +11867,7 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>1180</v>
+        <v>6</v>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
@@ -11900,7 +11900,7 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>1180</v>
+        <v>6</v>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
@@ -42547,11 +42547,11 @@
         </is>
       </c>
       <c r="D6" s="3">
-        <f>ROUND(0.15 * E5, 0)</f>
+        <f>ROUND(0.20 * E5, 0)</f>
         <v/>
       </c>
       <c r="E6" s="9">
-        <f>ROUND(0.15 * E5, 0)</f>
+        <f>ROUND(0.20 * E5, 0)</f>
         <v/>
       </c>
       <c r="F6" s="10">
@@ -42576,11 +42576,11 @@
         </is>
       </c>
       <c r="D7" s="2">
-        <f>ROUND(0.06 * (E5 + E6), 0)</f>
+        <f>ROUND(0.055 * (E5 + E6), 0)</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>ROUND(0.06 * (E5 + E6), 0)</f>
+        <f>ROUND(0.055 * (E5 + E6), 0)</f>
         <v/>
       </c>
       <c r="F7" s="8">
@@ -42605,11 +42605,11 @@
         </is>
       </c>
       <c r="D8" s="3">
-        <f>ROUND(0.05 * (E5 + E6 + E7), 0)</f>
+        <f>ROUND(0.00 * (E5 + E6 + E7), 0)</f>
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>ROUND(0.05 * (E5 + E6 + E7), 0)</f>
+        <f>ROUND(0.00 * (E5 + E6 + E7), 0)</f>
         <v/>
       </c>
       <c r="F8" s="10">

</xml_diff>